<commit_message>
push final code changes
</commit_message>
<xml_diff>
--- a/CW Testing.xlsx
+++ b/CW Testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1197bf129f5fe9f/Desktop/Birbeck/Cloud Computing/CW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{BABBBDA5-4C99-46BC-8145-AFFE94EBE183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6843D50-FC6E-4BCE-896D-B8CE5B7793C9}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="8_{BABBBDA5-4C99-46BC-8145-AFFE94EBE183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE88BA1B-2B0A-4D97-A087-C1C1FF39296A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F031067B-CAA1-421E-BF36-43FC9B0760DE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{F031067B-CAA1-421E-BF36-43FC9B0760DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Tests" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="78">
   <si>
     <t>Olga, Nick, Mary, and Nestor register and are ready to access the Piazza API.</t>
   </si>
@@ -774,7 +774,7 @@
         <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
@@ -788,7 +788,7 @@
         <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.35">
@@ -915,8 +915,11 @@
         <v>10</v>
       </c>
       <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="E16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B17" s="2" t="s">
         <v>18</v>
       </c>
@@ -924,8 +927,11 @@
         <v>77</v>
       </c>
       <c r="D17" s="3"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="E17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="2" t="s">
         <v>19</v>
       </c>
@@ -933,8 +939,11 @@
         <v>11</v>
       </c>
       <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="E18" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B19" s="2" t="s">
         <v>20</v>
       </c>
@@ -942,8 +951,11 @@
         <v>28</v>
       </c>
       <c r="D19" s="3"/>
-    </row>
-    <row r="20" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>21</v>
       </c>
@@ -951,8 +963,11 @@
         <v>29</v>
       </c>
       <c r="D20" s="3"/>
-    </row>
-    <row r="21" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="E20" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B21" s="2" t="s">
         <v>22</v>
       </c>
@@ -960,8 +975,11 @@
         <v>12</v>
       </c>
       <c r="D21" s="3"/>
-    </row>
-    <row r="22" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="E21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B22" s="2" t="s">
         <v>23</v>
       </c>
@@ -969,6 +987,9 @@
         <v>30</v>
       </c>
       <c r="D22" s="3"/>
+      <c r="E22" t="s">
+        <v>72</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>